<commit_message>
update(ai): re run tft_inference.ipynb
</commit_message>
<xml_diff>
--- a/data/predicted/tft_future_prediction_results.xlsx
+++ b/data/predicted/tft_future_prediction_results.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,10 +452,15 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>y3_future_pred</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>y4_future_pred</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>y5_future_pred</t>
         </is>
@@ -466,16 +471,19 @@
         <v>45839</v>
       </c>
       <c r="B2" t="n">
-        <v>21.53188705444336</v>
+        <v>23.58548545837402</v>
       </c>
       <c r="C2" t="n">
-        <v>26.12485122680664</v>
+        <v>28.9954948425293</v>
       </c>
       <c r="D2" t="n">
-        <v>27.27869033813477</v>
+        <v>1157.676391601562</v>
       </c>
       <c r="E2" t="n">
-        <v>9.016681671142578</v>
+        <v>25.36433792114258</v>
+      </c>
+      <c r="F2" t="n">
+        <v>11.70039176940918</v>
       </c>
     </row>
     <row r="3">
@@ -483,16 +491,19 @@
         <v>45839.04166666666</v>
       </c>
       <c r="B3" t="n">
-        <v>24.02226638793945</v>
+        <v>31.64772796630859</v>
       </c>
       <c r="C3" t="n">
-        <v>26.10272216796875</v>
+        <v>40.76568603515625</v>
       </c>
       <c r="D3" t="n">
-        <v>23.83525276184082</v>
+        <v>1190.903076171875</v>
       </c>
       <c r="E3" t="n">
-        <v>9.026745796203613</v>
+        <v>35.78872299194336</v>
+      </c>
+      <c r="F3" t="n">
+        <v>12.32982635498047</v>
       </c>
     </row>
     <row r="4">
@@ -500,16 +511,19 @@
         <v>45839.08333333334</v>
       </c>
       <c r="B4" t="n">
-        <v>26.49612808227539</v>
+        <v>40.96712112426758</v>
       </c>
       <c r="C4" t="n">
-        <v>29.75337982177734</v>
+        <v>49.16006088256836</v>
       </c>
       <c r="D4" t="n">
-        <v>31.23298263549805</v>
+        <v>2130.438232421875</v>
       </c>
       <c r="E4" t="n">
-        <v>11.52140998840332</v>
+        <v>35.46988677978516</v>
+      </c>
+      <c r="F4" t="n">
+        <v>15.72394275665283</v>
       </c>
     </row>
     <row r="5">
@@ -517,16 +531,19 @@
         <v>45839.125</v>
       </c>
       <c r="B5" t="n">
-        <v>36.72113800048828</v>
+        <v>28.53542900085449</v>
       </c>
       <c r="C5" t="n">
-        <v>30.44438743591309</v>
+        <v>31.10919761657715</v>
       </c>
       <c r="D5" t="n">
-        <v>33.7913818359375</v>
+        <v>1288.250732421875</v>
       </c>
       <c r="E5" t="n">
-        <v>11.83513355255127</v>
+        <v>33.01534652709961</v>
+      </c>
+      <c r="F5" t="n">
+        <v>21.38189506530762</v>
       </c>
     </row>
     <row r="6">
@@ -534,16 +551,19 @@
         <v>45839.16666666666</v>
       </c>
       <c r="B6" t="n">
-        <v>30.94128608703613</v>
+        <v>21.93515586853027</v>
       </c>
       <c r="C6" t="n">
-        <v>35.80070495605469</v>
+        <v>27.09988784790039</v>
       </c>
       <c r="D6" t="n">
-        <v>34.36314392089844</v>
+        <v>709.5691528320312</v>
       </c>
       <c r="E6" t="n">
-        <v>12.40752029418945</v>
+        <v>20.7646427154541</v>
+      </c>
+      <c r="F6" t="n">
+        <v>22.17016220092773</v>
       </c>
     </row>
     <row r="7">
@@ -551,16 +571,19 @@
         <v>45839.20833333334</v>
       </c>
       <c r="B7" t="n">
-        <v>38.26072311401367</v>
+        <v>17.07205581665039</v>
       </c>
       <c r="C7" t="n">
-        <v>37.14735794067383</v>
+        <v>38.23245620727539</v>
       </c>
       <c r="D7" t="n">
-        <v>31.13593292236328</v>
+        <v>411.9109497070312</v>
       </c>
       <c r="E7" t="n">
-        <v>11.214524269104</v>
+        <v>14.32086849212646</v>
+      </c>
+      <c r="F7" t="n">
+        <v>33.21524047851562</v>
       </c>
     </row>
     <row r="8">
@@ -568,16 +591,19 @@
         <v>45839.25</v>
       </c>
       <c r="B8" t="n">
-        <v>36.58241653442383</v>
+        <v>18.86838340759277</v>
       </c>
       <c r="C8" t="n">
-        <v>33.06634902954102</v>
+        <v>26.28741264343262</v>
       </c>
       <c r="D8" t="n">
-        <v>60.78096771240234</v>
+        <v>492.3324890136719</v>
       </c>
       <c r="E8" t="n">
-        <v>10.96525859832764</v>
+        <v>12.34754753112793</v>
+      </c>
+      <c r="F8" t="n">
+        <v>39.31234359741211</v>
       </c>
     </row>
     <row r="9">
@@ -585,16 +611,19 @@
         <v>45839.29166666666</v>
       </c>
       <c r="B9" t="n">
-        <v>39.7327880859375</v>
+        <v>18.10180473327637</v>
       </c>
       <c r="C9" t="n">
-        <v>49.43485641479492</v>
+        <v>32.40463638305664</v>
       </c>
       <c r="D9" t="n">
-        <v>39.37890625</v>
+        <v>461.67333984375</v>
       </c>
       <c r="E9" t="n">
-        <v>14.61349010467529</v>
+        <v>8.201038360595703</v>
+      </c>
+      <c r="F9" t="n">
+        <v>26.00113296508789</v>
       </c>
     </row>
     <row r="10">
@@ -602,16 +631,19 @@
         <v>45839.33333333334</v>
       </c>
       <c r="B10" t="n">
-        <v>20.70538711547852</v>
+        <v>15.66726207733154</v>
       </c>
       <c r="C10" t="n">
-        <v>29.75106430053711</v>
+        <v>22.66076850891113</v>
       </c>
       <c r="D10" t="n">
-        <v>37.54462051391602</v>
+        <v>443.16259765625</v>
       </c>
       <c r="E10" t="n">
-        <v>16.03999137878418</v>
+        <v>9.004433631896973</v>
+      </c>
+      <c r="F10" t="n">
+        <v>24.35012245178223</v>
       </c>
     </row>
     <row r="11">
@@ -619,16 +651,19 @@
         <v>45839.375</v>
       </c>
       <c r="B11" t="n">
-        <v>26.10182571411133</v>
+        <v>16.85386276245117</v>
       </c>
       <c r="C11" t="n">
-        <v>25.00902557373047</v>
+        <v>27.92352294921875</v>
       </c>
       <c r="D11" t="n">
-        <v>11.2619800567627</v>
+        <v>418.6710205078125</v>
       </c>
       <c r="E11" t="n">
-        <v>14.7656946182251</v>
+        <v>8.762564659118652</v>
+      </c>
+      <c r="F11" t="n">
+        <v>29.87432098388672</v>
       </c>
     </row>
     <row r="12">
@@ -636,16 +671,19 @@
         <v>45839.41666666666</v>
       </c>
       <c r="B12" t="n">
-        <v>13.63766860961914</v>
+        <v>23.53836059570312</v>
       </c>
       <c r="C12" t="n">
-        <v>25.33887100219727</v>
+        <v>21.67664337158203</v>
       </c>
       <c r="D12" t="n">
-        <v>11.42907428741455</v>
+        <v>447.2808227539062</v>
       </c>
       <c r="E12" t="n">
-        <v>14.01595592498779</v>
+        <v>12.51328372955322</v>
+      </c>
+      <c r="F12" t="n">
+        <v>29.37785911560059</v>
       </c>
     </row>
     <row r="13">
@@ -653,16 +691,19 @@
         <v>45839.45833333334</v>
       </c>
       <c r="B13" t="n">
-        <v>16.93289375305176</v>
+        <v>18.02101707458496</v>
       </c>
       <c r="C13" t="n">
-        <v>23.22795677185059</v>
+        <v>23.72617340087891</v>
       </c>
       <c r="D13" t="n">
-        <v>12.2612361907959</v>
+        <v>506.221923828125</v>
       </c>
       <c r="E13" t="n">
-        <v>13.74717044830322</v>
+        <v>8.267812728881836</v>
+      </c>
+      <c r="F13" t="n">
+        <v>18.43574333190918</v>
       </c>
     </row>
   </sheetData>

</xml_diff>